<commit_message>
feat: Add 3 Legal Risk Defense Modules (Fire Hazard Conflict Detector, Structural Video Record Manager, Weather Stop-Work Trigger) - 57 tests pass
</commit_message>
<xml_diff>
--- a/secure_local_data/콘크리트_품질관리대장.xlsx
+++ b/secure_local_data/콘크리트_품질관리대장.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -782,6 +782,70 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>CONC-20260829-05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026.08.29</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>지하 2층 바닥 슬래브 1구역</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>25-24-150</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2026.09.05</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>77.1%</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>2026.09.26</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>109.2%</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>28일 강도 적합 (PASS)</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>감리원 입회 타설 (누적 320m3)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Support dynamic local data directory override via Construct_DATA_DIR env variable
</commit_message>
<xml_diff>
--- a/secure_local_data/콘크리트_품질관리대장.xlsx
+++ b/secure_local_data/콘크리트_품질관리대장.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -846,6 +846,70 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>CONC-20260829-06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026.08.29</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>지하 2층 바닥 슬래브 1구역</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>25-24-150</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>2026.09.05</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>77.1%</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>2026.09.26</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>109.2%</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>28일 강도 적합 (PASS)</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>감리원 입회 타설 (누적 320m3)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add SHA-256 Content-Hash Caching and Daily Log Session Append/Merge (60 tests pass)
</commit_message>
<xml_diff>
--- a/secure_local_data/콘크리트_품질관리대장.xlsx
+++ b/secure_local_data/콘크리트_품질관리대장.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -910,6 +910,70 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>CONC-20260829-07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026.08.29</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>지하 2층 바닥 슬래브 1구역</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>25-24-150</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026.09.05</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>77.1%</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>2026.09.26</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>109.2%</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>28일 강도 적합 (PASS)</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>감리원 입회 타설 (누적 320m3)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: enrich proposal with SAI RAG comparison, 1-on-1 personal agent, MCP extensibility, and GitHub link
</commit_message>
<xml_diff>
--- a/secure_local_data/콘크리트_품질관리대장.xlsx
+++ b/secure_local_data/콘크리트_품질관리대장.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -974,6 +974,198 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>CONC-20260829-08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026.08.29</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>지하 2층 바닥 슬래브 1구역</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>25-24-150</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2026.09.05</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>77.1%</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>2026.09.26</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>109.2%</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>28일 강도 적합 (PASS)</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>입력 자료 기반 등록</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>CONC-20260829-09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026.08.29</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>지하 2층 바닥 슬래브 1구역</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>25-24-150</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026.09.05</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>77.1%</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>2026.09.26</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>109.2%</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>28일 강도 적합 (PASS)</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>입력 자료 기반 등록</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>CONC-20260829-10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026.08.29</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>지하 2층 바닥 슬래브 1구역</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>25-24-150</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2026.09.05</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>77.1%</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>2026.09.26</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>109.2%</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>28일 강도 적합 (PASS)</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>입력 자료 기반 등록</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>